<commit_message>
Reading new xlsx format, improved base_collectoin
</commit_message>
<xml_diff>
--- a/workspaces/example_new_calculations/input/settings.xlsx
+++ b/workspaces/example_new_calculations/input/settings.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKL\Documents\Github\GeoProb-Pipe\workspaces\example_new_calculations\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F41B3AF-CBD2-456D-8039-CB43EDBA810F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B94D10D-DB32-4DCB-93CD-1274631D6FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3A9227AB-5B1B-4583-A938-7605F1717FF5}"/>
+    <workbookView xWindow="28695" yWindow="5175" windowWidth="17280" windowHeight="8880" xr2:uid="{3A9227AB-5B1B-4583-A938-7605F1717FF5}"/>
   </bookViews>
   <sheets>
-    <sheet name="settings" sheetId="1" r:id="rId1"/>
+    <sheet name="Settings" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>